<commit_message>
ECS-98 added extended classifiers options in evaluation-logs-report-template.xlsx, classifiers-configuration-report-template.xlsx
</commit_message>
<xml_diff>
--- a/eca-server/src/main/resources/report-templates/classifiers-configuration-report-template.xlsx
+++ b/eca-server/src/main/resources/report-templates/classifiers-configuration-report-template.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8196" tabRatio="500"/>
@@ -11,7 +11,7 @@
     <sheet name="Лист2" sheetId="2" r:id="rId2"/>
     <sheet name="Лист3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="125725" iterateDelta="1E-4"/>
+  <calcPr calcId="124519" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -140,9 +140,6 @@
     <t>Классификатор</t>
   </si>
   <si>
-    <t>Настройки классификатора</t>
-  </si>
-  <si>
     <t>Конфигурация ${report.configurationName}</t>
   </si>
   <si>
@@ -173,9 +170,6 @@
     <t>Дата создания настроек</t>
   </si>
   <si>
-    <t>${classifierOptions.optionsName}</t>
-  </si>
-  <si>
     <t>${classifierOptions.config}</t>
   </si>
   <si>
@@ -189,6 +183,37 @@
   </si>
   <si>
     <t>ACTIVE</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">${classifierOptions.optionsName}
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+      </rPr>
+      <t>Настройки классификатора:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve">
+${classifierOptions.optionsString}</t>
+    </r>
+  </si>
+  <si>
+    <t>Настройки классификатора JSON</t>
   </si>
 </sst>
 </file>
@@ -308,7 +333,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
@@ -327,6 +352,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -706,12 +734,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.6">
-      <c r="A1" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
+      <c r="A1" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
@@ -720,7 +748,7 @@
     </row>
     <row r="2" spans="1:9" ht="15.6">
       <c r="A2" s="12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -733,7 +761,7 @@
     </row>
     <row r="3" spans="1:9" s="4" customFormat="1" ht="15.6">
       <c r="A3" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -746,10 +774,10 @@
     </row>
     <row r="4" spans="1:9" s="4" customFormat="1">
       <c r="A4" s="10" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -761,10 +789,10 @@
     </row>
     <row r="5" spans="1:9" s="4" customFormat="1">
       <c r="A5" s="10" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -776,10 +804,10 @@
     </row>
     <row r="6" spans="1:9" s="4" customFormat="1">
       <c r="A6" s="10" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -791,10 +819,10 @@
     </row>
     <row r="7" spans="1:9" s="4" customFormat="1">
       <c r="A7" s="10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -831,13 +859,13 @@
         <v>0</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
@@ -845,18 +873,18 @@
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
     </row>
-    <row r="11" spans="1:9">
-      <c r="A11" s="7" t="s">
+    <row r="11" spans="1:9" ht="14.4" customHeight="1">
+      <c r="A11" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="D11" s="7" t="s">
         <v>13</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>15</v>
       </c>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>

</xml_diff>